<commit_message>
docs: standardize Vietnamese P2P case study baseline
</commit_message>
<xml_diff>
--- a/02-stakeholder-analysis/P2P_Stakeholder_Register.xlsx
+++ b/02-stakeholder-analysis/P2P_Stakeholder_Register.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\AppData\Local\Temp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\retail-p2p-ba-case-study\02-stakeholder-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE433A3-C65F-4EB0-BA39-061474BD74AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DB0796-5A38-462C-B1BD-1840C3BCD835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,8 +18,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stakeholder Register'!$A$7:$G$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Influence-Interest Matrix'!$A$1:$E$8</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Stakeholder Register'!$A$1:$G$18</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -42,22 +44,22 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="99">
   <si>
-    <t>Procure-to-Pay (P2P) System Implementation</t>
-  </si>
-  <si>
-    <t>Stakeholder Register &amp; Engagement Matrix (Section 3)</t>
-  </si>
-  <si>
-    <t>TOTAL STAKEHOLDERS</t>
-  </si>
-  <si>
-    <t>HIGH INFLUENCE</t>
-  </si>
-  <si>
-    <t>HIGH INTEREST</t>
-  </si>
-  <si>
-    <t>EXTERNAL ENTITIES</t>
+    <t>Nghiên cứu tình huống phân tích nghiệp vụ (BA) quy trình mua hàng đến thanh toán (P2P)</t>
+  </si>
+  <si>
+    <t>Danh sách và ma trận phối hợp các bên liên quan (Stakeholder) — Đường cơ sở giả lập; chưa được các bên liên quan ký duyệt</t>
+  </si>
+  <si>
+    <t>TỔNG SỐ BÊN LIÊN QUAN</t>
+  </si>
+  <si>
+    <t>ẢNH HƯỞNG CAO</t>
+  </si>
+  <si>
+    <t>QUAN TÂM CAO</t>
+  </si>
+  <si>
+    <t>ĐƠN VỊ BÊN NGOÀI</t>
   </si>
   <si>
     <t>1</t>
@@ -66,277 +68,277 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Stakeholder</t>
-  </si>
-  <si>
-    <t>Role in P2P</t>
-  </si>
-  <si>
-    <t>Main Responsibilities</t>
-  </si>
-  <si>
-    <t>Main Needs / Expectations</t>
-  </si>
-  <si>
-    <t>Influence</t>
-  </si>
-  <si>
-    <t>Interest</t>
+    <t>Bên liên quan</t>
+  </si>
+  <si>
+    <t>Vai trò trong P2P</t>
+  </si>
+  <si>
+    <t>Trách nhiệm chính</t>
+  </si>
+  <si>
+    <t>Nhu cầu / Kỳ vọng chính</t>
+  </si>
+  <si>
+    <t>Mức ảnh hưởng</t>
+  </si>
+  <si>
+    <t>Mức quan tâm</t>
   </si>
   <si>
     <t>STK-01</t>
   </si>
   <si>
-    <t>Store Employee / Requester</t>
-  </si>
-  <si>
-    <t>Purchase requester</t>
-  </si>
-  <si>
-    <t>Identify purchasing needs, create and submit PR</t>
-  </si>
-  <si>
-    <t>Simple PR creation, clear status tracking, fewer manual steps</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>High</t>
+    <t>Nhân viên cửa hàng / Người yêu cầu</t>
+  </si>
+  <si>
+    <t>Người yêu cầu mua hàng</t>
+  </si>
+  <si>
+    <t>Xác định nhu cầu mua hàng, tạo và gửi yêu cầu mua hàng (PR)</t>
+  </si>
+  <si>
+    <t>Tạo PR đơn giản, theo dõi trạng thái rõ ràng, giảm bước thủ công</t>
+  </si>
+  <si>
+    <t>Thấp</t>
+  </si>
+  <si>
+    <t>Cao</t>
   </si>
   <si>
     <t>STK-02</t>
   </si>
   <si>
-    <t>Store Manager</t>
-  </si>
-  <si>
-    <t>Business approver / Cost owner</t>
-  </si>
-  <si>
-    <t>Review business need and approve or reject PR</t>
-  </si>
-  <si>
-    <t>Clear request information, budget visibility, fast approval process</t>
-  </si>
-  <si>
-    <t>Medium</t>
+    <t>Quản lý cửa hàng</t>
+  </si>
+  <si>
+    <t>Người phê duyệt nghiệp vụ / Chủ thể chịu trách nhiệm chi phí</t>
+  </si>
+  <si>
+    <t>Xem xét nhu cầu nghiệp vụ; phê duyệt, từ chối hoặc trả PR để chỉnh sửa</t>
+  </si>
+  <si>
+    <t>Thông tin yêu cầu rõ ràng, nắm được ngân sách, phê duyệt nhanh</t>
+  </si>
+  <si>
+    <t>Trung bình</t>
   </si>
   <si>
     <t>STK-03</t>
   </si>
   <si>
-    <t>Procurement Officer</t>
-  </si>
-  <si>
-    <t>Buyer / Operational procurement user</t>
-  </si>
-  <si>
-    <t>Review approved PR, select approved supplier, create and manage PO</t>
-  </si>
-  <si>
-    <t>Centralized information, reduced duplicate entry, clear workflow</t>
+    <t>Nhân viên mua hàng</t>
+  </si>
+  <si>
+    <t>Nhân viên thu mua / Người dùng nghiệp vụ mua hàng</t>
+  </si>
+  <si>
+    <t>Xem xét PR đã phê duyệt, chọn nhà cung cấp đã phê duyệt, tạo và quản lý đơn đặt hàng (PO)</t>
+  </si>
+  <si>
+    <t>Thông tin tập trung, giảm nhập trùng, luồng xử lý rõ ràng</t>
   </si>
   <si>
     <t>STK-04</t>
   </si>
   <si>
-    <t>Procurement Manager</t>
-  </si>
-  <si>
-    <t>Procurement Process Owner</t>
-  </si>
-  <si>
-    <t>Oversee procurement activities, enforce procurement rules, participate in PO approval</t>
-  </si>
-  <si>
-    <t>Process control, approval visibility, procurement KPIs</t>
+    <t>Trưởng bộ phận mua hàng</t>
+  </si>
+  <si>
+    <t>Chủ quy trình mua hàng</t>
+  </si>
+  <si>
+    <t>Giám sát mua hàng, thực thi quy tắc, thực hiện phê duyệt mua hàng bắt buộc cho mọi PO</t>
+  </si>
+  <si>
+    <t>Kiểm soát quy trình, theo dõi phê duyệt, chỉ số hiệu quả mua hàng (KPI)</t>
   </si>
   <si>
     <t>STK-05</t>
   </si>
   <si>
-    <t>Warehouse Staff</t>
-  </si>
-  <si>
-    <t>Goods receiver</t>
-  </si>
-  <si>
-    <t>Receive goods and record Goods Receipt</t>
-  </si>
-  <si>
-    <t>Clear PO reference, simple receipt recording, discrepancy capture</t>
+    <t>Nhân viên kho</t>
+  </si>
+  <si>
+    <t>Người nhận hàng</t>
+  </si>
+  <si>
+    <t>Nhận hàng và ghi nhận phiếu nhận hàng (GR)</t>
+  </si>
+  <si>
+    <t>Tham chiếu PO rõ ràng, ghi nhận nhận hàng đơn giản, ghi nhận sai lệch</t>
   </si>
   <si>
     <t>STK-06</t>
   </si>
   <si>
-    <t>AP Accountant</t>
-  </si>
-  <si>
-    <t>Invoice processing user</t>
-  </si>
-  <si>
-    <t>Record supplier invoices, perform 3-way matching, investigate mismatches</t>
-  </si>
-  <si>
-    <t>Accurate PO/GR data, automated matching, clear exception workflow</t>
+    <t>Kế toán công nợ phải trả (AP)</t>
+  </si>
+  <si>
+    <t>Người xử lý hóa đơn</t>
+  </si>
+  <si>
+    <t>Ghi nhận hóa đơn nhà cung cấp, thực hiện đối chiếu ba bên, điều tra sai lệch</t>
+  </si>
+  <si>
+    <t>Dữ liệu PO/GR chính xác, đối chiếu tự động, luồng xử lý ngoại lệ rõ ràng</t>
   </si>
   <si>
     <t>STK-07</t>
   </si>
   <si>
-    <t>Finance Manager</t>
-  </si>
-  <si>
-    <t>Financial Control Owner</t>
-  </si>
-  <si>
-    <t>Oversee budget control, financial approval and payment approval</t>
-  </si>
-  <si>
-    <t>Budget compliance, financial visibility, transaction traceability</t>
+    <t>Trưởng bộ phận tài chính</t>
+  </si>
+  <si>
+    <t>Chủ thể chịu trách nhiệm kiểm soát tài chính</t>
+  </si>
+  <si>
+    <t>Chịu trách nhiệm chính sách ngân sách, phê duyệt tài chính bổ sung cho PO và phê duyệt đề nghị thanh toán</t>
+  </si>
+  <si>
+    <t>Tuân thủ ngân sách, nắm được thông tin tài chính, truy vết giao dịch</t>
   </si>
   <si>
     <t>STK-08</t>
   </si>
   <si>
-    <t>CFO</t>
-  </si>
-  <si>
-    <t>Executive Sponsor</t>
-  </si>
-  <si>
-    <t>Provide sponsorship and oversee financial governance</t>
-  </si>
-  <si>
-    <t>Cost control, process performance, compliance and reliable reporting</t>
+    <t>Giám đốc tài chính (CFO)</t>
+  </si>
+  <si>
+    <t>Nhà bảo trợ cấp điều hành</t>
+  </si>
+  <si>
+    <t>Bảo trợ và giám sát quản trị tài chính</t>
+  </si>
+  <si>
+    <t>Kiểm soát chi phí, hiệu quả quy trình, tuân thủ và báo cáo đáng tin cậy</t>
   </si>
   <si>
     <t>STK-09</t>
   </si>
   <si>
-    <t>Internal Audit</t>
-  </si>
-  <si>
-    <t>Governance stakeholder</t>
-  </si>
-  <si>
-    <t>Review process controls and transaction history</t>
-  </si>
-  <si>
-    <t>Complete audit trail, segregation of duties and evidence of approval</t>
+    <t>Kiểm toán nội bộ</t>
+  </si>
+  <si>
+    <t>Bên liên quan về quản trị</t>
+  </si>
+  <si>
+    <t>Rà soát kiểm soát quy trình và lịch sử giao dịch</t>
+  </si>
+  <si>
+    <t>Dấu vết kiểm toán đầy đủ, phân tách nhiệm vụ và bằng chứng phê duyệt</t>
   </si>
   <si>
     <t>STK-10</t>
   </si>
   <si>
-    <t>IT Team</t>
-  </si>
-  <si>
-    <t>Supporting stakeholder</t>
-  </si>
-  <si>
-    <t>Support system implementation, access control and integration</t>
-  </si>
-  <si>
-    <t>Stable requirements, clear integration boundaries and maintainability</t>
+    <t>Bộ phận công nghệ thông tin (IT)</t>
+  </si>
+  <si>
+    <t>Bên liên quan hỗ trợ</t>
+  </si>
+  <si>
+    <t>Hỗ trợ triển khai hệ thống, kiểm soát truy cập và tích hợp</t>
+  </si>
+  <si>
+    <t>Yêu cầu ổn định, ranh giới tích hợp rõ ràng và khả năng bảo trì</t>
   </si>
   <si>
     <t>STK-11</t>
   </si>
   <si>
-    <t>Supplier</t>
-  </si>
-  <si>
-    <t>External business stakeholder</t>
-  </si>
-  <si>
-    <t>Receive PO, deliver goods and provide supplier invoice</t>
-  </si>
-  <si>
-    <t>Accurate PO information, clear communication and timely processing</t>
-  </si>
-  <si>
-    <t>Stakeholder Power / Interest Grid (Engagement Strategy)</t>
-  </si>
-  <si>
-    <t>Standard classification mapping for P2P project management governance</t>
-  </si>
-  <si>
-    <t>Quadrant</t>
-  </si>
-  <si>
-    <t>Strategy</t>
-  </si>
-  <si>
-    <t>Influence / Interest</t>
-  </si>
-  <si>
-    <t>P2P Stakeholders Included</t>
-  </si>
-  <si>
-    <t>Key Action</t>
-  </si>
-  <si>
-    <t>Manage Closely (Key Players)</t>
-  </si>
-  <si>
-    <t>High Influence, High Interest</t>
-  </si>
-  <si>
-    <t>High / High</t>
-  </si>
-  <si>
-    <t>STK-04 (Procurement Manager), STK-07 (Finance Manager)</t>
-  </si>
-  <si>
-    <t>Engage deeply in solution design, process approvals, and UAT sign-off.</t>
-  </si>
-  <si>
-    <t>Keep Satisfied</t>
-  </si>
-  <si>
-    <t>High Influence, Medium/Low Interest</t>
-  </si>
-  <si>
-    <t>High / Medium</t>
-  </si>
-  <si>
-    <t>STK-08 (CFO)</t>
-  </si>
-  <si>
-    <t>Provide concise executive dashboards, budget impact metrics, and milestone reports.</t>
-  </si>
-  <si>
-    <t>Keep Informed</t>
-  </si>
-  <si>
-    <t>Low Influence, High Interest</t>
-  </si>
-  <si>
-    <t>Low/Med / High</t>
-  </si>
-  <si>
-    <t>STK-01 (Requester), STK-02 (Store Mgr), STK-03 (Buyer), STK-05 (Warehouse), STK-06 (AP)</t>
-  </si>
-  <si>
-    <t>Provide hands-on training, interactive walkthroughs, and clear transition guidelines.</t>
-  </si>
-  <si>
-    <t>Monitor (Minimum Effort)</t>
-  </si>
-  <si>
-    <t>Low Influence, Low/Med Interest</t>
-  </si>
-  <si>
-    <t>Low/Med / Med</t>
-  </si>
-  <si>
-    <t>STK-09 (Audit), STK-10 (IT Team), STK-11 (Supplier)</t>
-  </si>
-  <si>
-    <t>Regular status briefings, API/system integration sync, and vendor onboarding kits.</t>
+    <t>Nhà cung cấp</t>
+  </si>
+  <si>
+    <t>Bên liên quan nghiệp vụ bên ngoài</t>
+  </si>
+  <si>
+    <t>Nhận PO, giao hàng và cung cấp hóa đơn nhà cung cấp</t>
+  </si>
+  <si>
+    <t>Thông tin PO chính xác, trao đổi rõ ràng và xử lý kịp thời</t>
+  </si>
+  <si>
+    <t>Ma trận mức ảnh hưởng / quan tâm của các bên liên quan (Chiến lược phối hợp)</t>
+  </si>
+  <si>
+    <t>Đề xuất phối hợp cho nghiên cứu tình huống BA; phân loại giả lập; chưa có ký duyệt của các bên liên quan</t>
+  </si>
+  <si>
+    <t>Nhóm trên ma trận</t>
+  </si>
+  <si>
+    <t>Chiến lược</t>
+  </si>
+  <si>
+    <t>Ảnh hưởng / Quan tâm</t>
+  </si>
+  <si>
+    <t>Các bên liên quan trong P2P</t>
+  </si>
+  <si>
+    <t>Hành động chính</t>
+  </si>
+  <si>
+    <t>Phối hợp chặt chẽ (Các bên chủ chốt)</t>
+  </si>
+  <si>
+    <t>Ảnh hưởng cao, quan tâm cao</t>
+  </si>
+  <si>
+    <t>Cao / Cao</t>
+  </si>
+  <si>
+    <t>STK-04 (Trưởng bộ phận mua hàng), STK-07 (Trưởng bộ phận tài chính)</t>
+  </si>
+  <si>
+    <t>Tham gia sâu vào thiết kế giải pháp, phê duyệt quy trình và ký duyệt kiểm thử chấp nhận người dùng (UAT).</t>
+  </si>
+  <si>
+    <t>Duy trì sự hài lòng</t>
+  </si>
+  <si>
+    <t>Ảnh hưởng cao, quan tâm trung bình/thấp</t>
+  </si>
+  <si>
+    <t>Cao / Trung bình</t>
+  </si>
+  <si>
+    <t>STK-08 (Giám đốc tài chính — CFO)</t>
+  </si>
+  <si>
+    <t>Cung cấp bảng tổng hợp ngắn gọn cho lãnh đạo, chỉ số tác động ngân sách và báo cáo mốc tiến độ.</t>
+  </si>
+  <si>
+    <t>Duy trì cung cấp thông tin</t>
+  </si>
+  <si>
+    <t>Ảnh hưởng thấp, quan tâm cao</t>
+  </si>
+  <si>
+    <t>Thấp/Trung bình / Cao</t>
+  </si>
+  <si>
+    <t>STK-01 (Người yêu cầu), STK-02 (Quản lý cửa hàng), STK-03 (Nhân viên mua hàng), STK-05 (Kho), STK-06 (AP)</t>
+  </si>
+  <si>
+    <t>Đào tạo thực hành, hướng dẫn từng bước có tương tác và hướng dẫn chuyển đổi rõ ràng.</t>
+  </si>
+  <si>
+    <t>Theo dõi (Mức nỗ lực tối thiểu)</t>
+  </si>
+  <si>
+    <t>Ảnh hưởng thấp, quan tâm thấp/trung bình</t>
+  </si>
+  <si>
+    <t>Thấp/Trung bình / Trung bình</t>
+  </si>
+  <si>
+    <t>STK-09 (Kiểm toán), STK-10 (IT), STK-11 (Nhà cung cấp)</t>
+  </si>
+  <si>
+    <t>Tham vấn Kiểm toán/IT theo nội dung cần thiết và trao đổi với nhà cung cấp đã phê duyệt về nhận PO, thông tin giao hàng và xử lý hóa đơn.</t>
   </si>
 </sst>
 </file>
@@ -493,78 +495,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,11 +577,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF008000"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -873,349 +873,352 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="5" width="44" customWidth="1"/>
-    <col min="6" max="7" width="14" customWidth="1"/>
+    <col min="1" max="1" width="11" style="7" customWidth="1"/>
+    <col min="2" max="2" width="28" style="7" customWidth="1"/>
+    <col min="3" max="3" width="32" style="7" customWidth="1"/>
+    <col min="4" max="5" width="44" style="7" customWidth="1"/>
+    <col min="6" max="7" width="14" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-    </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+    </row>
+    <row r="2" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-    </row>
-    <row r="4" spans="1:7" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+    </row>
+    <row r="4" spans="1:7" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="15" t="s">
+      <c r="B4" s="20"/>
+      <c r="C4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="15" t="s">
+      <c r="D4" s="20"/>
+      <c r="E4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="16"/>
-    </row>
-    <row r="5" spans="1:7" s="22" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="18">
+      <c r="G4" s="20"/>
+    </row>
+    <row r="5" spans="1:7" s="8" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="22">
         <f>COUNTA(A8:A18)</f>
         <v>11</v>
       </c>
       <c r="B5" s="23"/>
-      <c r="C5" s="18">
-        <f>COUNTIF(F8:F18, "High")</f>
+      <c r="C5" s="22">
+        <f>COUNTIF(F8:F18, "Cao")</f>
         <v>3</v>
       </c>
       <c r="D5" s="23"/>
-      <c r="E5" s="18">
-        <f>COUNTIF(G8:G18, "High")</f>
+      <c r="E5" s="22">
+        <f>COUNTIF(G8:G18, "Cao")</f>
         <v>7</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="22" t="s">
         <v>6</v>
       </c>
       <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:7" ht="9.6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:7" s="24" customFormat="1" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
+    <row r="7" spans="1:7" s="9" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="G7" s="10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+    <row r="9" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="F9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+    <row r="13" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="15" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+    <row r="17" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="G17" s="15" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="85.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="17" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1234,121 +1237,125 @@
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="8" orientation="landscape"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
+    <col min="1" max="1" width="28" style="7" customWidth="1"/>
+    <col min="2" max="2" width="24" style="7" customWidth="1"/>
+    <col min="3" max="3" width="18" style="7" customWidth="1"/>
+    <col min="4" max="4" width="38" style="7" customWidth="1"/>
+    <col min="5" max="5" width="46" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-    </row>
-    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+    </row>
+    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-    </row>
-    <row r="4" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+    </row>
+    <row r="4" spans="1:5" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="18" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:5" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:5" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:5" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="4" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:5" ht="109.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1358,5 +1365,6 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="8" orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>